<commit_message>
added fact sheets per board and rig
</commit_message>
<xml_diff>
--- a/surf_equipment.xlsx
+++ b/surf_equipment.xlsx
@@ -19,144 +19,162 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId15" roundtripDataChecksum="p6BhCJO34hERBBZVxSJO2AALWp4FAT5ZshcPml/zI9I="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId15" roundtripDataChecksum="RLbXDDqPLJ2eE0UZ5jO3FdYDo92Kn9VezziuKRng0bo="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="164">
+  <si>
+    <t>mast_id</t>
+  </si>
   <si>
     <t>sail_id</t>
   </si>
   <si>
-    <t>mast_id</t>
+    <t>length</t>
+  </si>
+  <si>
+    <t>area</t>
+  </si>
+  <si>
+    <t>diameter</t>
+  </si>
+  <si>
+    <t>discipline</t>
+  </si>
+  <si>
+    <t>carbon_perc</t>
   </si>
   <si>
     <t>extension_id</t>
   </si>
   <si>
-    <t>area</t>
-  </si>
-  <si>
-    <t>length</t>
+    <t>curve</t>
+  </si>
+  <si>
+    <t>mast_length</t>
+  </si>
+  <si>
+    <t>bag</t>
+  </si>
+  <si>
+    <t>mast_diameter_ind</t>
   </si>
   <si>
     <t>brand</t>
   </si>
   <si>
-    <t>discipline</t>
-  </si>
-  <si>
-    <t>diameter</t>
+    <t>mast_curve_ind</t>
+  </si>
+  <si>
+    <t>model</t>
+  </si>
+  <si>
+    <t>color</t>
   </si>
   <si>
     <t>origin</t>
   </si>
   <si>
-    <t>mast_length</t>
+    <t>boom_length_ind</t>
+  </si>
+  <si>
+    <t>400 SDM</t>
+  </si>
+  <si>
+    <t>Prolomit</t>
+  </si>
+  <si>
+    <t>cambers</t>
   </si>
   <si>
     <t>base_pulley_id</t>
   </si>
   <si>
-    <t>carbon_perc</t>
-  </si>
-  <si>
-    <t>mast_diameter_ind</t>
-  </si>
-  <si>
-    <t>curve</t>
-  </si>
-  <si>
-    <t>mast_curve_ind</t>
-  </si>
-  <si>
-    <t>Prolomit</t>
+    <t>Prolimit</t>
+  </si>
+  <si>
+    <t>SDM</t>
   </si>
   <si>
     <t>length_range</t>
   </si>
   <si>
-    <t>boom_length_ind</t>
-  </si>
-  <si>
-    <t>bag</t>
-  </si>
-  <si>
-    <t>model</t>
-  </si>
-  <si>
-    <t>cambers</t>
-  </si>
-  <si>
-    <t>color</t>
-  </si>
-  <si>
-    <t>Prolimit</t>
-  </si>
-  <si>
     <t>Beginner's sail</t>
   </si>
   <si>
+    <t>J&amp;J</t>
+  </si>
+  <si>
+    <t>freeride</t>
+  </si>
+  <si>
+    <t>SDM/RDM</t>
+  </si>
+  <si>
+    <t>cc</t>
+  </si>
+  <si>
+    <t>157-161</t>
+  </si>
+  <si>
+    <t>no</t>
+  </si>
+  <si>
+    <t>STX</t>
+  </si>
+  <si>
+    <t>Arrows</t>
+  </si>
+  <si>
+    <t>?</t>
+  </si>
+  <si>
+    <t>white</t>
+  </si>
+  <si>
+    <t>400 RDM</t>
+  </si>
+  <si>
+    <t>blue/orange</t>
+  </si>
+  <si>
+    <t>Etienne</t>
+  </si>
+  <si>
+    <t>RDM</t>
+  </si>
+  <si>
+    <t>Freek</t>
+  </si>
+  <si>
     <t>Short pulley</t>
   </si>
   <si>
-    <t>400 SDM</t>
-  </si>
-  <si>
-    <t>J&amp;J</t>
-  </si>
-  <si>
-    <t>freeride</t>
+    <t>Duotone</t>
+  </si>
+  <si>
+    <t>Gold</t>
+  </si>
+  <si>
+    <t>gold/white</t>
+  </si>
+  <si>
+    <t>freestyle</t>
   </si>
   <si>
     <t>n.a.</t>
   </si>
   <si>
-    <t>SDM/RDM</t>
-  </si>
-  <si>
-    <t>cc</t>
-  </si>
-  <si>
-    <t>SDM</t>
-  </si>
-  <si>
-    <t>157-161</t>
-  </si>
-  <si>
-    <t>?</t>
-  </si>
-  <si>
-    <t>Arrows</t>
-  </si>
-  <si>
-    <t>no</t>
-  </si>
-  <si>
-    <t>blue/orange</t>
-  </si>
-  <si>
-    <t>Etienne</t>
-  </si>
-  <si>
-    <t>Freek</t>
-  </si>
-  <si>
-    <t>freestyle</t>
-  </si>
-  <si>
     <t>RDM only</t>
   </si>
   <si>
     <t>Severne</t>
   </si>
   <si>
-    <t>STX</t>
-  </si>
-  <si>
     <t>red</t>
   </si>
   <si>
@@ -166,57 +184,54 @@
     <t>Pilot</t>
   </si>
   <si>
-    <t>white</t>
+    <t>460-40</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>North Sails</t>
+  </si>
+  <si>
+    <t>RDM pulley</t>
   </si>
   <si>
     <t>Gaasta</t>
   </si>
   <si>
-    <t>RDM pulley</t>
-  </si>
-  <si>
-    <t>400 RDM</t>
+    <t>etienne</t>
+  </si>
+  <si>
+    <t>460-80</t>
   </si>
   <si>
     <t>blue/green</t>
   </si>
   <si>
-    <t>RDM</t>
-  </si>
-  <si>
     <t>Camber</t>
   </si>
   <si>
+    <t>Apex Pro</t>
+  </si>
+  <si>
+    <t>slalom</t>
+  </si>
+  <si>
     <t>Tiki</t>
   </si>
   <si>
-    <t>slalom</t>
-  </si>
-  <si>
-    <t>Duotone</t>
-  </si>
-  <si>
     <t>SDM only</t>
   </si>
   <si>
-    <t>Gold</t>
-  </si>
-  <si>
     <t>207-210</t>
   </si>
   <si>
-    <t>gold/white</t>
+    <t>Alu short pulley</t>
   </si>
   <si>
     <t>Neil Pryde</t>
   </si>
   <si>
-    <t>Alu short pulley</t>
-  </si>
-  <si>
-    <t>yes</t>
-  </si>
-  <si>
     <t>?-30</t>
   </si>
   <si>
@@ -235,39 +250,24 @@
     <t>Alu large pulley</t>
   </si>
   <si>
+    <t>?-45</t>
+  </si>
+  <si>
     <t>NCX</t>
   </si>
   <si>
-    <t>?-45</t>
-  </si>
-  <si>
     <t>Unifiber</t>
   </si>
   <si>
-    <t>460-40</t>
-  </si>
-  <si>
     <t>Chique pulley</t>
   </si>
   <si>
     <t>?-48</t>
   </si>
   <si>
-    <t>North Sails</t>
-  </si>
-  <si>
     <t>UXT</t>
   </si>
   <si>
-    <t>etienne</t>
-  </si>
-  <si>
-    <t>460-80</t>
-  </si>
-  <si>
-    <t>Apex Pro</t>
-  </si>
-  <si>
     <t>boom_id</t>
   </si>
   <si>
@@ -304,12 +304,18 @@
     <t>STX4</t>
   </si>
   <si>
+    <t>rdm_sdm_shim_id</t>
+  </si>
+  <si>
     <t>162-222</t>
   </si>
   <si>
     <t>4.0</t>
   </si>
   <si>
+    <t>The Shim</t>
+  </si>
+  <si>
     <t>STX2</t>
   </si>
   <si>
@@ -325,36 +331,30 @@
     <t>Technowind</t>
   </si>
   <si>
-    <t>rdm_sdm_shim_id</t>
-  </si>
-  <si>
-    <t>The Shim</t>
-  </si>
-  <si>
     <t>uphaul_id</t>
   </si>
   <si>
     <t>Black uphaul 1</t>
   </si>
   <si>
+    <t>Black uphaul 2</t>
+  </si>
+  <si>
+    <t>Yellow uphaul</t>
+  </si>
+  <si>
+    <t>yellow</t>
+  </si>
+  <si>
+    <t>Black uphaul 3</t>
+  </si>
+  <si>
     <t>harness_line_id</t>
   </si>
   <si>
-    <t>Black uphaul 2</t>
-  </si>
-  <si>
     <t>White harness line 1</t>
   </si>
   <si>
-    <t>Yellow uphaul</t>
-  </si>
-  <si>
-    <t>yellow</t>
-  </si>
-  <si>
-    <t>Black uphaul 3</t>
-  </si>
-  <si>
     <t>Hose</t>
   </si>
   <si>
@@ -373,85 +373,124 @@
     <t>board_id</t>
   </si>
   <si>
+    <t>story</t>
+  </si>
+  <si>
     <t>volume</t>
   </si>
   <si>
+    <t>vin</t>
+  </si>
+  <si>
+    <t>daggerboard</t>
+  </si>
+  <si>
+    <t>The Ship</t>
+  </si>
+  <si>
+    <t>The Ship got its name from its size: with 205 liter it's a very stable board on which you could easily organize a small party. It was once bought from Wim Ang of WVOP after an up-side down bidding process: Wim asked 100 euros for it. Since this felt almost as fencing, our counter-bid was 150 euros and we had a deal. When we bought it, the board was quite slippery. That was resolved by putting a thin layer of epoxy on it, and sprinkling some sugar on it. After the epoxy hardened, we threw the board into the water. The sugar resolved and a left a surface that feels like comfortably granular grinding paper. So you won't easily fall from The Ship. It even behaves well above 18 knots, since the 100 liter in the front are not used then as they are completely out of the water. Of course the primary purpose of this board is giving an easy entrance for beginners to the wonderful world of windsurfing. The secondary purpose is to offer experienced windsurfers complete guarantee for not falling into the water. This is very handy in case you don't have time to change clothes before windsuring and have to windsurf in your business suit with your telephone still in your pocket. This board has the nice feature that it has two fins. It also features an optional daggerboard for better upwind performance. We do not recommend to use The Ship with the ultralight rig. Every other rig works perfectly well on this board. Although The Ship could be used as a SUP as well, we don't recommend this becasue windsurfing is so much more fun!</t>
+  </si>
+  <si>
+    <t>Bic</t>
+  </si>
+  <si>
+    <t>Windfinder</t>
+  </si>
+  <si>
+    <t>beige (2x)</t>
+  </si>
+  <si>
+    <t>pink (optional)</t>
+  </si>
+  <si>
+    <t>Wim</t>
+  </si>
+  <si>
+    <t>Kode</t>
+  </si>
+  <si>
+    <t>Starboard</t>
+  </si>
+  <si>
+    <t>light green</t>
+  </si>
+  <si>
+    <t>black (optional)</t>
+  </si>
+  <si>
+    <t>Topsurf</t>
+  </si>
+  <si>
+    <t>Atomiq</t>
+  </si>
+  <si>
+    <t>dark green</t>
+  </si>
+  <si>
+    <t>Telstar</t>
+  </si>
+  <si>
+    <t>Nash</t>
+  </si>
+  <si>
+    <t>Robby Nash</t>
+  </si>
+  <si>
+    <t>Freeride</t>
+  </si>
+  <si>
+    <t>Black project or Wave 22</t>
+  </si>
+  <si>
+    <t>Haarlem</t>
+  </si>
+  <si>
     <t>rig_id</t>
   </si>
   <si>
-    <t>'t Schip</t>
-  </si>
-  <si>
-    <t>R1</t>
-  </si>
-  <si>
-    <t>Bic</t>
-  </si>
-  <si>
-    <t>Windfinder</t>
-  </si>
-  <si>
-    <t>Wim</t>
-  </si>
-  <si>
-    <t>Kode</t>
-  </si>
-  <si>
-    <t>Starboard</t>
-  </si>
-  <si>
-    <t>Topsurf</t>
-  </si>
-  <si>
-    <t>R2</t>
-  </si>
-  <si>
-    <t>Atomiq</t>
-  </si>
-  <si>
-    <t>Telstar</t>
-  </si>
-  <si>
-    <t>R3</t>
-  </si>
-  <si>
-    <t>Nash</t>
-  </si>
-  <si>
-    <t>Robby Nash</t>
-  </si>
-  <si>
-    <t>Freeride</t>
-  </si>
-  <si>
-    <t>Haarlem</t>
-  </si>
-  <si>
-    <t>R4</t>
-  </si>
-  <si>
-    <t>R5</t>
+    <t>base_pulley_lenght_setting</t>
   </si>
   <si>
     <t>rig_board_id</t>
   </si>
   <si>
+    <t>extension_length_setting</t>
+  </si>
+  <si>
     <t>RB01</t>
   </si>
   <si>
+    <t>boom_length_setting</t>
+  </si>
+  <si>
+    <t>Beginner's rig</t>
+  </si>
+  <si>
     <t>RB02</t>
   </si>
   <si>
+    <t>Pilot rig</t>
+  </si>
+  <si>
     <t>RB03</t>
   </si>
   <si>
+    <t>Camber rig</t>
+  </si>
+  <si>
     <t>RB04</t>
   </si>
   <si>
+    <t>8 meter rig</t>
+  </si>
+  <si>
     <t>RB05</t>
   </si>
   <si>
     <t>RB06</t>
+  </si>
+  <si>
+    <t>Ultralight rig</t>
   </si>
   <si>
     <t>RB07</t>
@@ -503,12 +542,12 @@
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Arial"/>
     </font>
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Aptos Narrow"/>
     </font>
   </fonts>
   <fills count="2">
@@ -525,7 +564,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -535,10 +574,10 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -548,11 +587,10 @@
       <alignment horizontal="left"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf quotePrefix="1" borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -816,229 +854,229 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>9</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>17</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>20</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B2" s="4">
+        <v>25</v>
+      </c>
+      <c r="B2" s="3">
         <v>4.7</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="3">
         <v>400.0</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F2" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="G2" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="I2" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="I2" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="K2" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="L2" s="3" t="s">
+      <c r="J2" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="K2" s="4" t="s">
         <v>37</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B3" s="4">
+        <v>40</v>
+      </c>
+      <c r="B3" s="3">
         <v>4.8</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="D3" s="4">
+      <c r="C3" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D3" s="3">
         <v>415.0</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="G3" s="6">
+        <v>161.0</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="I3" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="F3" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="G3" s="5">
-        <v>161.0</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="L3" s="4" t="s">
+      <c r="J3" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="L3" s="3" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="B4" s="4">
+        <v>51</v>
+      </c>
+      <c r="B4" s="3">
         <v>6.5</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="3">
         <v>430.0</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F4" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="F4" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="G4" s="5">
+      <c r="G4" s="6">
         <v>195.0</v>
       </c>
-      <c r="H4" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="K4" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="L4" s="4" t="s">
+      <c r="H4" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="L4" s="3" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B5" s="4">
+        <v>60</v>
+      </c>
+      <c r="B5" s="3">
         <v>7.0</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="D5" s="4">
+      <c r="C5" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="D5" s="3">
         <v>490.0</v>
       </c>
-      <c r="E5" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="K5" s="3" t="s">
+      <c r="E5" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="L5" s="3" t="s">
-        <v>37</v>
+      <c r="F5" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="L5" s="4" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="B6" s="4">
+        <v>70</v>
+      </c>
+      <c r="B6" s="3">
         <v>8.0</v>
       </c>
-      <c r="C6" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="D6" s="4">
+      <c r="C6" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="D6" s="3">
         <v>460.0</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="F6" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="G6" s="5">
+      <c r="G6" s="6">
         <v>200.0</v>
       </c>
-      <c r="H6" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="I6" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="J6" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="K6" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="L6" s="4" t="s">
+      <c r="H6" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="L6" s="3" t="s">
         <v>26</v>
       </c>
     </row>
@@ -1058,150 +1096,180 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
   <cols>
     <col customWidth="1" min="4" max="4" width="13.25"/>
-    <col customWidth="1" min="7" max="7" width="16.0"/>
+    <col customWidth="1" min="9" max="10" width="16.0"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="D1" s="1" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>2</v>
+        <v>140</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="I1" s="1" t="s">
-        <v>103</v>
+      <c r="L1" s="1" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>118</v>
+        <v>145</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>15</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="E2" s="2"/>
       <c r="F2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>125</v>
+        <v>154</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>49</v>
+        <v>36</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="F3" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="G3" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>105</v>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="C4" s="2">
         <v>430.0</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="F4" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="H4" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="I4" s="2" t="s">
+      <c r="K4" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="L4" s="2" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>133</v>
+        <v>149</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>72</v>
-      </c>
       <c r="D5" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>105</v>
+        <v>73</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>134</v>
+        <v>151</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>78</v>
+        <v>58</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="I6" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="L6" s="2" t="s">
         <v>113</v>
       </c>
     </row>
@@ -1219,178 +1287,178 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>114</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="s">
-        <v>136</v>
+      <c r="A2" s="8" t="s">
+        <v>143</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>118</v>
+        <v>145</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="s">
-        <v>137</v>
+      <c r="A3" s="8" t="s">
+        <v>146</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="s">
-        <v>138</v>
+      <c r="A4" s="8" t="s">
+        <v>148</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>133</v>
+        <v>149</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="s">
-        <v>139</v>
+      <c r="A5" s="8" t="s">
+        <v>150</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="10" t="s">
-        <v>140</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>122</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="10" t="s">
-        <v>141</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="10" t="s">
-        <v>142</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="10" t="s">
-        <v>143</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="10" t="s">
-        <v>144</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="10" t="s">
-        <v>145</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="10" t="s">
-        <v>146</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>126</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="10" t="s">
-        <v>147</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>126</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="10" t="s">
-        <v>148</v>
-      </c>
-      <c r="B14" s="9" t="s">
-        <v>126</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="10" t="s">
-        <v>149</v>
-      </c>
-      <c r="B15" s="9" t="s">
-        <v>126</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="10" t="s">
-        <v>150</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>129</v>
-      </c>
       <c r="C16" s="1" t="s">
-        <v>125</v>
+        <v>154</v>
       </c>
     </row>
   </sheetData>
@@ -1413,97 +1481,97 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>7</v>
-      </c>
       <c r="D1" s="1" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B2" s="4">
+        <v>18</v>
+      </c>
+      <c r="B2" s="3">
         <v>400.0</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="5">
+        <v>20.0</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="F2" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D2" s="6">
-        <v>20.0</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H2" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I2" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="G2" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="I2" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="J2" s="3" t="s">
+      <c r="J2" s="4" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B3" s="4">
+        <v>36</v>
+      </c>
+      <c r="B3" s="3">
         <v>400.0</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="D3" s="3">
+      <c r="C3" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D3" s="4">
         <v>90.0</v>
       </c>
-      <c r="E3" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>55</v>
+      <c r="E3" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>42</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="J3" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="J3" s="4" t="s">
         <v>26</v>
       </c>
     </row>
@@ -1511,95 +1579,95 @@
       <c r="A4" s="2">
         <v>430.0</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="3">
         <v>430.0</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="5">
+        <v>20.0</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D4" s="6">
-        <v>20.0</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="F4" s="3" t="s">
+      <c r="G4" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I4" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="G4" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="J4" s="3" t="s">
+      <c r="J4" s="4" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="B5" s="4">
+        <v>52</v>
+      </c>
+      <c r="B5" s="3">
         <v>460.0</v>
       </c>
-      <c r="C5" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="D5" s="6">
+      <c r="C5" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" s="5">
         <v>40.0</v>
       </c>
-      <c r="E5" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>75</v>
+      <c r="E5" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>54</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>77</v>
+        <v>34</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="B6" s="4">
+        <v>58</v>
+      </c>
+      <c r="B6" s="3">
         <v>460.0</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="D6" s="6">
+      <c r="C6" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="5">
         <v>80.0</v>
       </c>
-      <c r="E6" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>41</v>
+      <c r="E6" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>48</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="I6" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="J6" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J6" s="4" t="s">
         <v>26</v>
       </c>
     </row>
@@ -1625,23 +1693,23 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B2" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>26</v>
       </c>
     </row>
@@ -1667,122 +1735,122 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>16</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>31</v>
+        <v>41</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>23</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="F2" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="F2" s="4" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>51</v>
+        <v>55</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>39</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="F3" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="F3" s="4" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>31</v>
+        <v>66</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>23</v>
       </c>
       <c r="D4" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="F4" s="3" t="s">
+      <c r="E4" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="F4" s="4" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>31</v>
+        <v>73</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>23</v>
       </c>
       <c r="D5" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="E5" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="E5" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="4" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>31</v>
+        <v>77</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>23</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>37</v>
+        <v>79</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -1825,16 +1893,16 @@
       <c r="A2" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="4" t="s">
         <v>26</v>
       </c>
     </row>
@@ -1842,68 +1910,68 @@
       <c r="A3" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>90</v>
       </c>
       <c r="C3" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="D3" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>37</v>
+      <c r="E3" s="4" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="D4" s="4" t="s">
+      <c r="B4" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="C4" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="E5" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="E5" s="3" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="C6" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>37</v>
+      <c r="B6" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -1928,21 +1996,21 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>44</v>
+        <v>95</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>50</v>
       </c>
       <c r="C2" s="7" t="s">
         <v>26</v>
@@ -1973,10 +2041,10 @@
         <v>101</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2">
@@ -1984,43 +2052,43 @@
         <v>102</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="C2" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="C3" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="C4" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>37</v>
+        <v>50</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -2045,21 +2113,21 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>46</v>
+        <v>108</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>35</v>
       </c>
       <c r="C2" s="7" t="s">
         <v>26</v>
@@ -2069,7 +2137,7 @@
       <c r="A3" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>110</v>
       </c>
       <c r="C3" s="7" t="s">
@@ -2080,8 +2148,8 @@
       <c r="A4" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>46</v>
+      <c r="B4" s="4" t="s">
+        <v>35</v>
       </c>
       <c r="C4" s="7" t="s">
         <v>26</v>
@@ -2091,11 +2159,11 @@
       <c r="A5" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>37</v>
+      <c r="B5" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -2113,9 +2181,9 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="2" width="8.63"/>
-    <col customWidth="1" min="3" max="3" width="11.63"/>
-    <col customWidth="1" min="4" max="27" width="8.63"/>
+    <col customWidth="1" min="1" max="3" width="8.63"/>
+    <col customWidth="1" min="4" max="4" width="11.63"/>
+    <col customWidth="1" min="5" max="30" width="8.63"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2126,81 +2194,116 @@
         <v>115</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>5</v>
+        <v>116</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>8</v>
+        <v>14</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="s">
-        <v>117</v>
-      </c>
-      <c r="B2" s="9">
+        <v>119</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="C2" s="9">
         <v>205.0</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>119</v>
-      </c>
       <c r="D2" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="s">
-        <v>122</v>
-      </c>
-      <c r="B3" s="9">
+        <v>126</v>
+      </c>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9">
         <v>137.0</v>
       </c>
-      <c r="C3" s="9" t="s">
-        <v>123</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>122</v>
+      <c r="D3" s="9" t="s">
+        <v>127</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>124</v>
+        <v>126</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="9" t="s">
-        <v>126</v>
-      </c>
-      <c r="B4" s="9">
+        <v>131</v>
+      </c>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9">
         <v>110.0</v>
       </c>
-      <c r="C4" s="9" t="s">
-        <v>123</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>126</v>
+      <c r="D4" s="9" t="s">
+        <v>127</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>127</v>
+        <v>131</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="s">
-        <v>129</v>
-      </c>
-      <c r="B5" s="9">
-        <v>80.0</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>130</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>131</v>
+        <v>134</v>
+      </c>
+      <c r="B5" s="9"/>
+      <c r="C5" s="1">
+        <v>90.0</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>135</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>132</v>
+        <v>136</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="16" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
solved rig_fact_sheet imperfections and some more
</commit_message>
<xml_diff>
--- a/surf_equipment.xlsx
+++ b/surf_equipment.xlsx
@@ -26,236 +26,248 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="168">
+  <si>
+    <t>sail_id</t>
+  </si>
+  <si>
+    <t>extension_id</t>
+  </si>
+  <si>
+    <t>area</t>
+  </si>
+  <si>
+    <t>discipline</t>
+  </si>
+  <si>
+    <t>brand</t>
+  </si>
+  <si>
+    <t>mast_length</t>
+  </si>
+  <si>
+    <t>origin</t>
+  </si>
+  <si>
+    <t>mast_diameter_ind</t>
+  </si>
+  <si>
+    <t>mast_curve_ind</t>
+  </si>
+  <si>
+    <t>Prolomit</t>
+  </si>
+  <si>
+    <t>boom_length_ind</t>
+  </si>
+  <si>
+    <t>model</t>
+  </si>
+  <si>
+    <t>Prolimit</t>
+  </si>
+  <si>
+    <t>J&amp;J</t>
+  </si>
+  <si>
+    <t>cambers</t>
+  </si>
+  <si>
+    <t>color</t>
+  </si>
+  <si>
+    <t>Beginner's sail</t>
+  </si>
+  <si>
+    <t>4.7</t>
+  </si>
+  <si>
+    <t>freeride</t>
+  </si>
+  <si>
+    <t>SDM/RDM</t>
+  </si>
+  <si>
+    <t>cc</t>
+  </si>
+  <si>
+    <t>157-161</t>
+  </si>
+  <si>
+    <t>Arrows</t>
+  </si>
+  <si>
+    <t>?</t>
+  </si>
+  <si>
+    <t>no</t>
+  </si>
+  <si>
+    <t>blue/orange</t>
+  </si>
+  <si>
+    <t>Etienne</t>
+  </si>
+  <si>
+    <t>Freek</t>
+  </si>
+  <si>
+    <t>4.8</t>
+  </si>
+  <si>
+    <t>freestyle</t>
+  </si>
+  <si>
+    <t>RDM only</t>
+  </si>
+  <si>
+    <t>Severne</t>
+  </si>
+  <si>
+    <t>red</t>
+  </si>
   <si>
     <t>mast_id</t>
   </si>
   <si>
-    <t>sail_id</t>
+    <t>Pilot</t>
+  </si>
+  <si>
+    <t>6.5</t>
   </si>
   <si>
     <t>length</t>
   </si>
   <si>
-    <t>area</t>
+    <t>Gaasta</t>
   </si>
   <si>
     <t>diameter</t>
   </si>
   <si>
-    <t>discipline</t>
+    <t>blue/green</t>
   </si>
   <si>
     <t>carbon_perc</t>
   </si>
   <si>
-    <t>extension_id</t>
+    <t>Camber</t>
+  </si>
+  <si>
+    <t>7.0</t>
   </si>
   <si>
     <t>curve</t>
   </si>
   <si>
-    <t>mast_length</t>
+    <t>slalom</t>
+  </si>
+  <si>
+    <t>SDM only</t>
   </si>
   <si>
     <t>bag</t>
   </si>
   <si>
-    <t>mast_diameter_ind</t>
-  </si>
-  <si>
-    <t>brand</t>
-  </si>
-  <si>
-    <t>mast_curve_ind</t>
-  </si>
-  <si>
-    <t>model</t>
-  </si>
-  <si>
-    <t>color</t>
-  </si>
-  <si>
-    <t>origin</t>
-  </si>
-  <si>
-    <t>boom_length_ind</t>
+    <t>207-210</t>
+  </si>
+  <si>
+    <t>Neil Pryde</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>orange</t>
+  </si>
+  <si>
+    <t>8 meter</t>
+  </si>
+  <si>
+    <t>8.0</t>
+  </si>
+  <si>
+    <t>freerace</t>
   </si>
   <si>
     <t>400 SDM</t>
   </si>
   <si>
-    <t>Prolomit</t>
-  </si>
-  <si>
-    <t>cambers</t>
+    <t>NCX</t>
+  </si>
+  <si>
+    <t>SDM</t>
+  </si>
+  <si>
+    <t>STX</t>
+  </si>
+  <si>
+    <t>white</t>
+  </si>
+  <si>
+    <t>400 RDM</t>
+  </si>
+  <si>
+    <t>RDM</t>
+  </si>
+  <si>
+    <t>Duotone</t>
+  </si>
+  <si>
+    <t>Gold</t>
+  </si>
+  <si>
+    <t>gold/white</t>
+  </si>
+  <si>
+    <t>460-40</t>
+  </si>
+  <si>
+    <t>North Sails</t>
+  </si>
+  <si>
+    <t>black</t>
+  </si>
+  <si>
+    <t>etienne</t>
   </si>
   <si>
     <t>base_pulley_id</t>
   </si>
   <si>
-    <t>Prolimit</t>
-  </si>
-  <si>
-    <t>SDM</t>
+    <t>460-80</t>
+  </si>
+  <si>
+    <t>Apex Pro</t>
   </si>
   <si>
     <t>length_range</t>
   </si>
   <si>
-    <t>Beginner's sail</t>
-  </si>
-  <si>
-    <t>J&amp;J</t>
-  </si>
-  <si>
-    <t>freeride</t>
-  </si>
-  <si>
-    <t>SDM/RDM</t>
-  </si>
-  <si>
-    <t>cc</t>
-  </si>
-  <si>
-    <t>157-161</t>
-  </si>
-  <si>
-    <t>no</t>
-  </si>
-  <si>
-    <t>STX</t>
-  </si>
-  <si>
-    <t>Arrows</t>
-  </si>
-  <si>
-    <t>?</t>
-  </si>
-  <si>
-    <t>white</t>
-  </si>
-  <si>
-    <t>400 RDM</t>
-  </si>
-  <si>
-    <t>blue/orange</t>
-  </si>
-  <si>
-    <t>Etienne</t>
-  </si>
-  <si>
-    <t>RDM</t>
-  </si>
-  <si>
-    <t>Freek</t>
-  </si>
-  <si>
     <t>Short pulley</t>
   </si>
   <si>
-    <t>Duotone</t>
-  </si>
-  <si>
-    <t>Gold</t>
-  </si>
-  <si>
-    <t>gold/white</t>
-  </si>
-  <si>
-    <t>freestyle</t>
-  </si>
-  <si>
-    <t>n.a.</t>
-  </si>
-  <si>
-    <t>RDM only</t>
-  </si>
-  <si>
-    <t>Severne</t>
-  </si>
-  <si>
-    <t>red</t>
-  </si>
-  <si>
-    <t>black</t>
-  </si>
-  <si>
-    <t>Pilot</t>
-  </si>
-  <si>
-    <t>460-40</t>
-  </si>
-  <si>
-    <t>yes</t>
-  </si>
-  <si>
-    <t>North Sails</t>
-  </si>
-  <si>
     <t>RDM pulley</t>
   </si>
   <si>
-    <t>Gaasta</t>
-  </si>
-  <si>
-    <t>etienne</t>
-  </si>
-  <si>
-    <t>460-80</t>
-  </si>
-  <si>
-    <t>blue/green</t>
-  </si>
-  <si>
-    <t>Camber</t>
-  </si>
-  <si>
-    <t>Apex Pro</t>
-  </si>
-  <si>
-    <t>slalom</t>
-  </si>
-  <si>
     <t>Tiki</t>
   </si>
   <si>
-    <t>SDM only</t>
-  </si>
-  <si>
-    <t>207-210</t>
-  </si>
-  <si>
     <t>Alu short pulley</t>
   </si>
   <si>
-    <t>Neil Pryde</t>
-  </si>
-  <si>
     <t>?-30</t>
   </si>
   <si>
-    <t>orange</t>
-  </si>
-  <si>
-    <t>8 meter</t>
-  </si>
-  <si>
     <t>alu</t>
   </si>
   <si>
-    <t>freerace</t>
-  </si>
-  <si>
     <t>Alu large pulley</t>
   </si>
   <si>
     <t>?-45</t>
   </si>
   <si>
-    <t>NCX</t>
-  </si>
-  <si>
     <t>Unifiber</t>
   </si>
   <si>
@@ -304,33 +316,33 @@
     <t>STX4</t>
   </si>
   <si>
+    <t>162-222</t>
+  </si>
+  <si>
+    <t>4.0</t>
+  </si>
+  <si>
+    <t>STX2</t>
+  </si>
+  <si>
+    <t>2.0</t>
+  </si>
+  <si>
+    <t>Italian boom</t>
+  </si>
+  <si>
+    <t>140-230</t>
+  </si>
+  <si>
+    <t>Technowind</t>
+  </si>
+  <si>
     <t>rdm_sdm_shim_id</t>
   </si>
   <si>
-    <t>162-222</t>
-  </si>
-  <si>
-    <t>4.0</t>
-  </si>
-  <si>
     <t>The Shim</t>
   </si>
   <si>
-    <t>STX2</t>
-  </si>
-  <si>
-    <t>2.0</t>
-  </si>
-  <si>
-    <t>Italian boom</t>
-  </si>
-  <si>
-    <t>140-230</t>
-  </si>
-  <si>
-    <t>Technowind</t>
-  </si>
-  <si>
     <t>uphaul_id</t>
   </si>
   <si>
@@ -346,12 +358,12 @@
     <t>yellow</t>
   </si>
   <si>
+    <t>harness_line_id</t>
+  </si>
+  <si>
     <t>Black uphaul 3</t>
   </si>
   <si>
-    <t>harness_line_id</t>
-  </si>
-  <si>
     <t>White harness line 1</t>
   </si>
   <si>
@@ -394,6 +406,9 @@
     <t>Bic</t>
   </si>
   <si>
+    <t>rig_id</t>
+  </si>
+  <si>
     <t>Windfinder</t>
   </si>
   <si>
@@ -412,24 +427,36 @@
     <t>Starboard</t>
   </si>
   <si>
+    <t>base_pulley_lenght_setting</t>
+  </si>
+  <si>
     <t>light green</t>
   </si>
   <si>
     <t>black (optional)</t>
   </si>
   <si>
+    <t>extension_length_setting</t>
+  </si>
+  <si>
     <t>Topsurf</t>
   </si>
   <si>
     <t>Atomiq</t>
   </si>
   <si>
+    <t>boom_length_setting</t>
+  </si>
+  <si>
     <t>dark green</t>
   </si>
   <si>
     <t>Telstar</t>
   </si>
   <si>
+    <t>Beginner's rig</t>
+  </si>
+  <si>
     <t>Nash</t>
   </si>
   <si>
@@ -445,52 +472,37 @@
     <t>Haarlem</t>
   </si>
   <si>
-    <t>rig_id</t>
-  </si>
-  <si>
-    <t>base_pulley_lenght_setting</t>
+    <t>Ultralight rig</t>
+  </si>
+  <si>
+    <t>Pilot rig</t>
+  </si>
+  <si>
+    <t>Camber rig</t>
+  </si>
+  <si>
+    <t>8 meter rig</t>
   </si>
   <si>
     <t>rig_board_id</t>
   </si>
   <si>
-    <t>extension_length_setting</t>
-  </si>
-  <si>
     <t>RB01</t>
   </si>
   <si>
-    <t>boom_length_setting</t>
-  </si>
-  <si>
-    <t>Beginner's rig</t>
-  </si>
-  <si>
     <t>RB02</t>
   </si>
   <si>
-    <t>Pilot rig</t>
-  </si>
-  <si>
     <t>RB03</t>
   </si>
   <si>
-    <t>Camber rig</t>
-  </si>
-  <si>
     <t>RB04</t>
   </si>
   <si>
-    <t>8 meter rig</t>
-  </si>
-  <si>
     <t>RB05</t>
   </si>
   <si>
     <t>RB06</t>
-  </si>
-  <si>
-    <t>Ultralight rig</t>
   </si>
   <si>
     <t>RB07</t>
@@ -542,12 +554,12 @@
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Aptos Narrow"/>
     </font>
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="2">
@@ -574,10 +586,10 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -587,7 +599,7 @@
       <alignment horizontal="left"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
@@ -854,230 +866,230 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>9</v>
-      </c>
       <c r="E1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>20</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>15</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" s="4">
+        <v>400.0</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K2" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="3">
-        <v>4.7</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="D2" s="3">
-        <v>400.0</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="G2" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>38</v>
+      <c r="L2" s="3" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="B3" s="3">
-        <v>4.8</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="D3" s="3">
+        <v>27</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D3" s="4">
         <v>415.0</v>
       </c>
-      <c r="E3" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="G3" s="6">
+      <c r="E3" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" s="5">
         <v>161.0</v>
       </c>
-      <c r="H3" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="J3" s="4" t="s">
+      <c r="H3" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="K3" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>26</v>
+      <c r="I3" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="B4" s="3">
-        <v>6.5</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="D4" s="3">
+        <v>34</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="4">
         <v>430.0</v>
       </c>
-      <c r="E4" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="G4" s="6">
+      <c r="E4" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G4" s="5">
         <v>195.0</v>
       </c>
-      <c r="H4" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="K4" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>26</v>
+      <c r="H4" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="L4" s="4" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="B5" s="3">
-        <v>7.0</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="D5" s="3">
+        <v>41</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D5" s="4">
         <v>490.0</v>
       </c>
-      <c r="E5" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="L5" s="4" t="s">
-        <v>38</v>
+      <c r="E5" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="B6" s="3">
-        <v>8.0</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="D6" s="3">
+        <v>51</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D6" s="4">
         <v>460.0</v>
       </c>
-      <c r="E6" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="G6" s="6">
+      <c r="E6" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G6" s="5">
         <v>200.0</v>
       </c>
-      <c r="H6" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="I6" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="J6" s="4" t="s">
+      <c r="H6" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="K6" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="L6" s="3" t="s">
-        <v>26</v>
+      <c r="I6" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="L6" s="4" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -1096,154 +1108,166 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
   <cols>
     <col customWidth="1" min="4" max="4" width="13.25"/>
+    <col customWidth="1" min="5" max="5" width="23.25"/>
     <col customWidth="1" min="9" max="10" width="16.0"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>144</v>
-      </c>
       <c r="J1" s="1" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>18</v>
+        <v>54</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>41</v>
+        <v>72</v>
       </c>
       <c r="E2" s="2"/>
       <c r="F2" s="2" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>85</v>
+        <v>89</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>23</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="G3" s="2"/>
       <c r="H3" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="I3" s="1"/>
+        <v>93</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>23</v>
+      </c>
       <c r="J3" s="1" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>51</v>
+        <v>34</v>
       </c>
       <c r="C4" s="2">
         <v>430.0</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="G4" s="2"/>
       <c r="H4" s="2" t="s">
-        <v>91</v>
+        <v>95</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>23</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="G5" s="2"/>
       <c r="H5" s="2" t="s">
-        <v>96</v>
+        <v>98</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>23</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
     </row>
     <row r="6">
@@ -1251,26 +1275,29 @@
         <v>151</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>70</v>
+        <v>51</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="G6" s="2"/>
       <c r="H6" s="2" t="s">
-        <v>98</v>
+        <v>100</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>23</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
     </row>
   </sheetData>
@@ -1287,54 +1314,54 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>141</v>
+        <v>152</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>139</v>
+        <v>126</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="s">
-        <v>143</v>
+        <v>153</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>151</v>
@@ -1342,54 +1369,54 @@
     </row>
     <row r="6">
       <c r="A6" s="8" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>151</v>
@@ -1397,54 +1424,54 @@
     </row>
     <row r="11">
       <c r="A11" s="8" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>151</v>
@@ -1452,13 +1479,13 @@
     </row>
     <row r="16">
       <c r="A16" s="8" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
     </row>
   </sheetData>
@@ -1481,194 +1508,194 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>2</v>
+        <v>36</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>12</v>
-      </c>
       <c r="H1" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>15</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B2" s="3">
+        <v>54</v>
+      </c>
+      <c r="B2" s="4">
         <v>400.0</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D2" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="H2" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="5">
-        <v>20.0</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>26</v>
+      <c r="I2" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B3" s="3">
+        <v>59</v>
+      </c>
+      <c r="B3" s="4">
         <v>400.0</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="D3" s="4">
+      <c r="C3" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D3" s="3">
         <v>90.0</v>
       </c>
-      <c r="E3" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>42</v>
+      <c r="E3" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>61</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>26</v>
+        <v>62</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2">
         <v>430.0</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="4">
         <v>430.0</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D4" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="H4" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="5">
-        <v>20.0</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>26</v>
+      <c r="I4" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B5" s="3">
+        <v>64</v>
+      </c>
+      <c r="B5" s="4">
         <v>460.0</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D5" s="6">
+        <v>40.0</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="H5" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="5">
-        <v>40.0</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>57</v>
+      <c r="I5" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="B6" s="3">
+        <v>69</v>
+      </c>
+      <c r="B6" s="4">
         <v>460.0</v>
       </c>
-      <c r="C6" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="D6" s="5">
+      <c r="C6" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D6" s="6">
         <v>80.0</v>
       </c>
-      <c r="E6" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>48</v>
+      <c r="E6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="I6" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="J6" s="4" t="s">
-        <v>26</v>
+        <v>70</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -1693,24 +1720,24 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>26</v>
+        <v>9</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -1735,122 +1762,120 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>21</v>
+        <v>68</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>24</v>
+        <v>71</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>4</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>12</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>15</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="C2" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D2" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>26</v>
+      <c r="E2" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>39</v>
+        <v>73</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>60</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>26</v>
+        <v>74</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>23</v>
+        <v>75</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>56</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>26</v>
+        <v>12</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>23</v>
+        <v>78</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>56</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>26</v>
+        <v>80</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>23</v>
+        <v>81</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>56</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>38</v>
+        <v>83</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -1874,104 +1899,104 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>26</v>
+        <v>89</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>90</v>
+        <v>93</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>94</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>38</v>
+        <v>23</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>26</v>
+        <v>95</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>26</v>
+      <c r="C5" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="C6" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="D6" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>38</v>
+      <c r="B6" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -1996,24 +2021,24 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>50</v>
+        <v>104</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>66</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -2038,57 +2063,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>26</v>
+        <v>66</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>26</v>
+        <v>66</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>26</v>
+        <v>109</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>38</v>
+        <v>66</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -2113,57 +2138,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>35</v>
+        <v>112</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>58</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>110</v>
+        <v>113</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>114</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>35</v>
+        <v>116</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>58</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>38</v>
+        <v>117</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -2188,122 +2213,128 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="C2" s="9">
         <v>205.0</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="s">
-        <v>126</v>
-      </c>
-      <c r="B3" s="9"/>
+        <v>131</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>23</v>
+      </c>
       <c r="C3" s="9">
         <v>137.0</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="B4" s="9"/>
+        <v>138</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>23</v>
+      </c>
       <c r="C4" s="9">
         <v>110.0</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="G4" s="1"/>
       <c r="H4" s="1" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="s">
-        <v>134</v>
-      </c>
-      <c r="B5" s="9"/>
+        <v>143</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>23</v>
+      </c>
       <c r="C5" s="1">
         <v>90.0</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G5" s="1"/>
       <c r="H5" s="1" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
     </row>
     <row r="16" ht="15.75" customHeight="1"/>

</xml_diff>